<commit_message>
fixed datasets: PDXE_v1, McGill_v2, UHN_lung_v1, UHN_breast_v1. consistant with orcestra and zenodo. re-extracted data and finalized numbers in figure 1.
</commit_message>
<xml_diff>
--- a/data/procdata/0_datasets/summary/dataset_summary.xlsx
+++ b/data/procdata/0_datasets/summary/dataset_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/guanqiaofeng/Documents/BHK/XevaDB/Manuscript_gitrepo/XevaDB_case_study/data/procdata/0_datasets/summary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CCFB982-5DDE-2346-B0B7-11FED976B84F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5D3EA81-C3AC-E840-A025-29393DB10B59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35600" yWindow="880" windowWidth="28040" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34560" yWindow="2140" windowWidth="29160" windowHeight="17420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -633,14 +633,14 @@
         <v>117</v>
       </c>
       <c r="D2">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E2">
         <v>277</v>
       </c>
       <c r="F2">
         <f t="shared" ref="F2:F8" si="0">SUM(B2:E2)</f>
-        <v>468</v>
+        <v>464</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -654,14 +654,14 @@
         <v>342</v>
       </c>
       <c r="D3">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E3">
         <v>277</v>
       </c>
       <c r="F3">
         <f t="shared" si="0"/>
-        <v>693</v>
+        <v>689</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -672,17 +672,17 @@
         <v>34</v>
       </c>
       <c r="C4">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D4">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E4">
         <v>277</v>
       </c>
       <c r="F4">
         <f t="shared" si="0"/>
-        <v>464</v>
+        <v>459</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -693,7 +693,7 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -703,7 +703,7 @@
       </c>
       <c r="F5">
         <f t="shared" si="0"/>
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -821,14 +821,14 @@
         <v>2683</v>
       </c>
       <c r="D11">
-        <v>1726</v>
+        <v>1415</v>
       </c>
       <c r="E11">
         <v>4706</v>
       </c>
       <c r="F11">
         <f>SUM(B11:E11)</f>
-        <v>9356</v>
+        <v>9045</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -842,14 +842,14 @@
         <v>1197</v>
       </c>
       <c r="D12">
-        <v>1156</v>
+        <v>914</v>
       </c>
       <c r="E12">
         <v>4483</v>
       </c>
       <c r="F12">
         <f>SUM(B12:E12)</f>
-        <v>7003</v>
+        <v>6761</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -863,14 +863,14 @@
         <v>1486</v>
       </c>
       <c r="D13">
-        <v>570</v>
+        <v>501</v>
       </c>
       <c r="E13">
         <v>223</v>
       </c>
       <c r="F13">
         <f>SUM(B13:E13)</f>
-        <v>2353</v>
+        <v>2284</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -884,14 +884,14 @@
         <v>594</v>
       </c>
       <c r="D14">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="E14">
         <v>3968</v>
       </c>
       <c r="F14">
         <f>SUM(B14:E14)</f>
-        <v>4852</v>
+        <v>4829</v>
       </c>
     </row>
   </sheetData>
@@ -960,7 +960,7 @@
         <v>48</v>
       </c>
       <c r="C5">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -1023,7 +1023,7 @@
         <v>30</v>
       </c>
       <c r="C11">
-        <v>715</v>
+        <v>689</v>
       </c>
     </row>
   </sheetData>

</xml_diff>